<commit_message>
feat: Introduce new odds scraping, PBP client, player impact and props engines, feature engineering v2, backtesting, and extensive new tests for data, models, and algorithms.
</commit_message>
<xml_diff>
--- a/results/nba_predictions_2025-12-13.xlsx
+++ b/results/nba_predictions_2025-12-13.xlsx
@@ -562,16 +562,16 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>47.27</v>
+        <v>52</v>
       </c>
       <c r="E2" t="n">
-        <v>52.73</v>
+        <v>48</v>
       </c>
       <c r="F2" t="n">
-        <v>56.44</v>
+        <v>56.4</v>
       </c>
       <c r="G2" t="n">
-        <v>43.56</v>
+        <v>43.6</v>
       </c>
       <c r="H2" t="n">
         <v>-0.15</v>
@@ -608,13 +608,13 @@
         <v>0</v>
       </c>
       <c r="R2" t="n">
-        <v>47.3</v>
+        <v>52</v>
       </c>
       <c r="S2" t="n">
-        <v>52.7</v>
+        <v>48</v>
       </c>
       <c r="T2" t="n">
-        <v>231.6</v>
+        <v>229.1</v>
       </c>
       <c r="U2" t="inlineStr">
         <is>
@@ -627,7 +627,7 @@
         </is>
       </c>
       <c r="W2" t="n">
-        <v>-1.6</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="3">
@@ -647,16 +647,16 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>63.89</v>
+        <v>52</v>
       </c>
       <c r="E3" t="n">
-        <v>36.11</v>
+        <v>48</v>
       </c>
       <c r="F3" t="n">
-        <v>58.93</v>
+        <v>58.97</v>
       </c>
       <c r="G3" t="n">
-        <v>41.07</v>
+        <v>41.03</v>
       </c>
       <c r="H3" t="n">
         <v>0.66</v>
@@ -678,7 +678,7 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
@@ -693,13 +693,13 @@
         <v>0</v>
       </c>
       <c r="R3" t="n">
-        <v>63.9</v>
+        <v>52</v>
       </c>
       <c r="S3" t="n">
-        <v>36.1</v>
+        <v>48</v>
       </c>
       <c r="T3" t="n">
-        <v>233.8</v>
+        <v>234.7</v>
       </c>
       <c r="U3" t="inlineStr">
         <is>
@@ -712,7 +712,7 @@
         </is>
       </c>
       <c r="W3" t="n">
-        <v>8.300000000000001</v>
+        <v>1.2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add OddsPedia web scraper with cache statistics and update changelog.
</commit_message>
<xml_diff>
--- a/results/nba_predictions_2025-12-13.xlsx
+++ b/results/nba_predictions_2025-12-13.xlsx
@@ -562,16 +562,16 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>52</v>
+        <v>40.38</v>
       </c>
       <c r="E2" t="n">
-        <v>48</v>
+        <v>59.62</v>
       </c>
       <c r="F2" t="n">
-        <v>56.4</v>
+        <v>56.46</v>
       </c>
       <c r="G2" t="n">
-        <v>43.6</v>
+        <v>43.54</v>
       </c>
       <c r="H2" t="n">
         <v>-0.15</v>
@@ -593,7 +593,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>MEDIUM</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -608,13 +608,13 @@
         <v>0</v>
       </c>
       <c r="R2" t="n">
-        <v>52</v>
+        <v>40.4</v>
       </c>
       <c r="S2" t="n">
-        <v>48</v>
+        <v>59.6</v>
       </c>
       <c r="T2" t="n">
-        <v>229.1</v>
+        <v>223.6</v>
       </c>
       <c r="U2" t="inlineStr">
         <is>
@@ -627,7 +627,7 @@
         </is>
       </c>
       <c r="W2" t="n">
-        <v>1.2</v>
+        <v>-5.8</v>
       </c>
     </row>
     <row r="3">
@@ -647,16 +647,16 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>52</v>
+        <v>55.1</v>
       </c>
       <c r="E3" t="n">
-        <v>48</v>
+        <v>44.9</v>
       </c>
       <c r="F3" t="n">
-        <v>58.97</v>
+        <v>58.96</v>
       </c>
       <c r="G3" t="n">
-        <v>41.03</v>
+        <v>41.04</v>
       </c>
       <c r="H3" t="n">
         <v>0.66</v>
@@ -678,7 +678,7 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>MEDIUM</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
@@ -693,13 +693,13 @@
         <v>0</v>
       </c>
       <c r="R3" t="n">
-        <v>52</v>
+        <v>55.1</v>
       </c>
       <c r="S3" t="n">
-        <v>48</v>
+        <v>44.9</v>
       </c>
       <c r="T3" t="n">
-        <v>234.7</v>
+        <v>227.4</v>
       </c>
       <c r="U3" t="inlineStr">
         <is>
@@ -712,7 +712,7 @@
         </is>
       </c>
       <c r="W3" t="n">
-        <v>1.2</v>
+        <v>3.1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>